<commit_message>
Taslak v2: AS3 temiz sozluk re-run (konusma 58->14%, uretim emergent; uydurma manset kaldirildi); APA duzeltme (Davar tam yazar, Jeon et al.); Appendix C sozlukler + duyarlilik; PRISMA 27-madde checklist
</commit_message>
<xml_diff>
--- a/projects/yz-yabancidil-derleme/analysis/bibliometric_tables.xlsx
+++ b/projects/yz-yabancidil-derleme/analysis/bibliometric_tables.xlsx
@@ -961,16 +961,16 @@
         <v>72</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>70.8</v>
+        <v>58.3</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>5.6</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="5">
@@ -983,16 +983,16 @@
         <v>246</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>39.4</v>
+        <v>35</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>20.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1005,16 +1005,16 @@
         <v>2732</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>606</v>
+        <v>391</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>22.2</v>
+        <v>14.3</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1037</v>
+        <v>31</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>38</v>
+        <v>1.1</v>
       </c>
     </row>
   </sheetData>
@@ -1289,7 +1289,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>affective backchannels</t>
+          <t>willingness to communicate in l2</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -1315,7 +1315,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>communication strategies</t>
+          <t>affective backchannels</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -1341,7 +1341,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>willingness to communicate in l2</t>
+          <t>communication strategies</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
@@ -1393,7 +1393,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>conversational technology</t>
+          <t>natural language visualization</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -1419,7 +1419,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>natural language visualization</t>
+          <t>conversational technology</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">

</xml_diff>